<commit_message>
fix: resolve reactive domain update on Home (HOME-018) and update QA docs
</commit_message>
<xml_diff>
--- a/Skillit_QA_Test_Report.xlsx
+++ b/Skillit_QA_Test_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/868af55b16e02466/Desktop/codes/extras/skillit-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_3F4C96BE085EF1FA77C6B918C4011D2484EEB7CA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85BF81E2-07E7-4165-B84A-EE3B99EC5E29}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_3F4C96BE085EF1FA77C6B918C4011D2484EEB7CA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA618568-A82F-4348-8418-A8C97102E25C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3311" uniqueCount="1060">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3271" uniqueCount="1060">
   <si>
     <t>SKILLIT</t>
   </si>
@@ -3218,7 +3218,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3419,6 +3419,12 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1A1A2E"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -3683,7 +3689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3955,6 +3961,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="41" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12374,7 +12386,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -12596,7 +12608,7 @@
       <c r="E9" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="93" t="s">
         <v>98</v>
       </c>
       <c r="G9" s="32" t="s">
@@ -12689,25 +12701,25 @@
         <v>35</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>118</v>
-      </c>
-      <c r="G13" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H13" s="33" t="s">
-        <v>68</v>
+        <v>129</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12715,25 +12727,25 @@
         <v>35</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>124</v>
-      </c>
-      <c r="G14" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H14" s="33" t="s">
-        <v>68</v>
+        <v>135</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12741,19 +12753,19 @@
         <v>35</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C15" s="30" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="G15" s="32" t="s">
         <v>67</v>
@@ -12767,19 +12779,19 @@
         <v>35</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G16" s="32" t="s">
         <v>67</v>
@@ -12793,25 +12805,25 @@
         <v>35</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="C17" s="30" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="G17" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H17" s="33" t="s">
-        <v>68</v>
+        <v>150</v>
+      </c>
+      <c r="G17" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12819,25 +12831,25 @@
         <v>35</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="G18" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="37" t="s">
-        <v>130</v>
+      <c r="H18" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12845,25 +12857,25 @@
         <v>35</v>
       </c>
       <c r="B19" s="39" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="G19" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H19" s="37" t="s">
-        <v>130</v>
+      <c r="H19" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12871,76 +12883,24 @@
         <v>35</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="G20" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H20" s="33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="39" t="s">
-        <v>156</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>159</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H21" s="33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="40" t="s">
-        <v>161</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>163</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>164</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>165</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" s="37" t="s">
+      <c r="H20" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -12949,12 +12909,13 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13196,7 +13157,7 @@
       <c r="C10" s="34" t="s">
         <v>202</v>
       </c>
-      <c r="D10" s="35" t="s">
+      <c r="D10" s="94" t="s">
         <v>203</v>
       </c>
       <c r="E10" s="35" t="s">
@@ -13216,72 +13177,72 @@
       <c r="A11" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="42" t="s">
-        <v>206</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>207</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>209</v>
-      </c>
-      <c r="F11" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="G11" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H11" s="33" t="s">
-        <v>68</v>
+      <c r="B11" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>212</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>213</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>214</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="43" t="s">
-        <v>211</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>212</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>213</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>214</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>215</v>
+      <c r="B12" s="42" t="s">
+        <v>216</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>219</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>220</v>
       </c>
       <c r="G12" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="37" t="s">
-        <v>130</v>
+      <c r="H12" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="42" t="s">
-        <v>216</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>217</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="E13" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="F13" s="31" t="s">
-        <v>220</v>
+      <c r="B13" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>222</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>223</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>224</v>
+      </c>
+      <c r="F13" s="35" t="s">
+        <v>225</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>67</v>
@@ -13294,20 +13255,20 @@
       <c r="A14" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="43" t="s">
-        <v>221</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>222</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>223</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>224</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>225</v>
+      <c r="B14" s="42" t="s">
+        <v>226</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>230</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>67</v>
@@ -13320,46 +13281,46 @@
       <c r="A15" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="42" t="s">
-        <v>226</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>228</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="F15" s="31" t="s">
-        <v>230</v>
+      <c r="B15" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>232</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>234</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>235</v>
       </c>
       <c r="G15" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="33" t="s">
-        <v>68</v>
+      <c r="H15" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="43" t="s">
-        <v>231</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>233</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>234</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>235</v>
+      <c r="B16" s="42" t="s">
+        <v>236</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>240</v>
       </c>
       <c r="G16" s="32" t="s">
         <v>67</v>
@@ -13372,72 +13333,72 @@
       <c r="A17" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="42" t="s">
-        <v>236</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>237</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>238</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>239</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>240</v>
+      <c r="B17" s="43" t="s">
+        <v>241</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>242</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>243</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>244</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>245</v>
       </c>
       <c r="G17" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="37" t="s">
-        <v>130</v>
+      <c r="H17" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>242</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>243</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>244</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>245</v>
+      <c r="B18" s="42" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>247</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>250</v>
       </c>
       <c r="G18" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="33" t="s">
-        <v>68</v>
+      <c r="H18" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="42" t="s">
-        <v>246</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>247</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>248</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>250</v>
+      <c r="B19" s="43" t="s">
+        <v>251</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>255</v>
       </c>
       <c r="G19" s="32" t="s">
         <v>67</v>
@@ -13450,23 +13411,23 @@
       <c r="A20" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="43" t="s">
-        <v>251</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>252</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>253</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>254</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>255</v>
-      </c>
-      <c r="G20" s="36" t="s">
-        <v>119</v>
+      <c r="B20" s="42" t="s">
+        <v>256</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>257</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>260</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H20" s="37" t="s">
         <v>130</v>
@@ -13476,51 +13437,25 @@
       <c r="A21" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="42" t="s">
-        <v>256</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>257</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>259</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>260</v>
+      <c r="B21" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>264</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>265</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>67</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B22" s="43" t="s">
-        <v>261</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>263</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>264</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>265</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -13529,12 +13464,13 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13900,23 +13836,23 @@
       <c r="A15" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="45" t="s">
-        <v>325</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>326</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>327</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>328</v>
-      </c>
-      <c r="F15" s="31" t="s">
-        <v>329</v>
-      </c>
-      <c r="G15" s="36" t="s">
-        <v>119</v>
+      <c r="B15" s="46" t="s">
+        <v>330</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>331</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>333</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>334</v>
+      </c>
+      <c r="G15" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H15" s="37" t="s">
         <v>130</v>
@@ -13926,20 +13862,20 @@
       <c r="A16" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="46" t="s">
-        <v>330</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>331</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>332</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>333</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>334</v>
+      <c r="B16" s="45" t="s">
+        <v>335</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>337</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>339</v>
       </c>
       <c r="G16" s="32" t="s">
         <v>67</v>
@@ -13952,20 +13888,20 @@
       <c r="A17" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="45" t="s">
-        <v>335</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>336</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>337</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>339</v>
+      <c r="B17" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>341</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>342</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>343</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>344</v>
       </c>
       <c r="G17" s="32" t="s">
         <v>67</v>
@@ -13978,20 +13914,20 @@
       <c r="A18" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="46" t="s">
-        <v>340</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>341</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>342</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>343</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>344</v>
+      <c r="B18" s="45" t="s">
+        <v>345</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>346</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>347</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>348</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>349</v>
       </c>
       <c r="G18" s="32" t="s">
         <v>67</v>
@@ -14004,23 +13940,23 @@
       <c r="A19" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="45" t="s">
-        <v>345</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>346</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>347</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>348</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>349</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>119</v>
+      <c r="B19" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>351</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>352</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>353</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>354</v>
+      </c>
+      <c r="G19" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H19" s="37" t="s">
         <v>130</v>
@@ -14030,20 +13966,20 @@
       <c r="A20" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="46" t="s">
-        <v>350</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>352</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>353</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>354</v>
+      <c r="B20" s="45" t="s">
+        <v>355</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>356</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>357</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>359</v>
       </c>
       <c r="G20" s="32" t="s">
         <v>67</v>
@@ -14056,51 +13992,25 @@
       <c r="A21" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="45" t="s">
-        <v>355</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>356</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>357</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>358</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>359</v>
+      <c r="B21" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>361</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>362</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>363</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>364</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>67</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="46" t="s">
-        <v>360</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>361</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>362</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>363</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>364</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -14114,7 +14024,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14194,75 +14104,75 @@
       <c r="A4" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="49" t="s">
-        <v>370</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>371</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>372</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>373</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>374</v>
-      </c>
-      <c r="G4" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H4" s="37" t="s">
-        <v>130</v>
+      <c r="B4" s="48" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>376</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>377</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>378</v>
+      </c>
+      <c r="F4" s="31" t="s">
+        <v>379</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="48" t="s">
-        <v>375</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>376</v>
-      </c>
-      <c r="D5" s="31" t="s">
-        <v>377</v>
-      </c>
-      <c r="E5" s="31" t="s">
-        <v>378</v>
-      </c>
-      <c r="F5" s="31" t="s">
-        <v>379</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H5" s="33" t="s">
-        <v>68</v>
+      <c r="B5" s="49" t="s">
+        <v>380</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>381</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>382</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>383</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>384</v>
+      </c>
+      <c r="G5" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H5" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="49" t="s">
-        <v>380</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>381</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>382</v>
-      </c>
-      <c r="E6" s="35" t="s">
-        <v>383</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>384</v>
-      </c>
-      <c r="G6" s="36" t="s">
-        <v>119</v>
+      <c r="B6" s="48" t="s">
+        <v>385</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>386</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>387</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>388</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>389</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H6" s="37" t="s">
         <v>130</v>
@@ -14272,46 +14182,46 @@
       <c r="A7" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="48" t="s">
-        <v>385</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>386</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>387</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>388</v>
-      </c>
-      <c r="F7" s="31" t="s">
-        <v>389</v>
+      <c r="B7" s="49" t="s">
+        <v>390</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>391</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>392</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>393</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>394</v>
       </c>
       <c r="G7" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="37" t="s">
-        <v>130</v>
+      <c r="H7" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="49" t="s">
-        <v>390</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>391</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>392</v>
-      </c>
-      <c r="E8" s="35" t="s">
-        <v>393</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>394</v>
+      <c r="B8" s="48" t="s">
+        <v>395</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>396</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>397</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>398</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>399</v>
       </c>
       <c r="G8" s="32" t="s">
         <v>67</v>
@@ -14324,46 +14234,46 @@
       <c r="A9" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="48" t="s">
-        <v>395</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>396</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>397</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>398</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>399</v>
+      <c r="B9" s="49" t="s">
+        <v>400</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>401</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>402</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>403</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>404</v>
       </c>
       <c r="G9" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H9" s="33" t="s">
-        <v>68</v>
+      <c r="H9" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>400</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>401</v>
-      </c>
-      <c r="D10" s="35" t="s">
-        <v>402</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>403</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>404</v>
+      <c r="B10" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>406</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>407</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>408</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>409</v>
       </c>
       <c r="G10" s="32" t="s">
         <v>67</v>
@@ -14376,72 +14286,72 @@
       <c r="A11" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="48" t="s">
-        <v>405</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>406</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>407</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>408</v>
-      </c>
-      <c r="F11" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="G11" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H11" s="37" t="s">
-        <v>130</v>
+      <c r="B11" s="49" t="s">
+        <v>410</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>411</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>412</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>413</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>414</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H11" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="49" t="s">
-        <v>410</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>411</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>412</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>413</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>414</v>
-      </c>
-      <c r="G12" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H12" s="33" t="s">
-        <v>68</v>
+      <c r="B12" s="48" t="s">
+        <v>415</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>416</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>417</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>418</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>419</v>
+      </c>
+      <c r="G12" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="48" t="s">
-        <v>415</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>416</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>417</v>
-      </c>
-      <c r="E13" s="31" t="s">
-        <v>418</v>
-      </c>
-      <c r="F13" s="31" t="s">
-        <v>419</v>
+      <c r="B13" s="49" t="s">
+        <v>420</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>421</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>422</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>423</v>
+      </c>
+      <c r="F13" s="35" t="s">
+        <v>424</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>67</v>
@@ -14454,20 +14364,20 @@
       <c r="A14" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="49" t="s">
-        <v>420</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>421</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>422</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>423</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>424</v>
+      <c r="B14" s="48" t="s">
+        <v>425</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>426</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>427</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>428</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>429</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>67</v>
@@ -14480,72 +14390,72 @@
       <c r="A15" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="48" t="s">
-        <v>425</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>426</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>427</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>428</v>
-      </c>
-      <c r="F15" s="31" t="s">
-        <v>429</v>
+      <c r="B15" s="49" t="s">
+        <v>430</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>431</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>432</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>434</v>
       </c>
       <c r="G15" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="37" t="s">
-        <v>130</v>
+      <c r="H15" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="49" t="s">
-        <v>430</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>431</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>432</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>433</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>434</v>
+      <c r="B16" s="48" t="s">
+        <v>435</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>436</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>437</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>438</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>439</v>
       </c>
       <c r="G16" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H16" s="33" t="s">
-        <v>68</v>
+      <c r="H16" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="48" t="s">
-        <v>435</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>436</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>437</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>438</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>439</v>
+      <c r="B17" s="49" t="s">
+        <v>440</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>441</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>442</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>443</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>444</v>
       </c>
       <c r="G17" s="32" t="s">
         <v>67</v>
@@ -14558,75 +14468,75 @@
       <c r="A18" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="49" t="s">
-        <v>440</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>441</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>442</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>443</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>444</v>
+      <c r="B18" s="48" t="s">
+        <v>445</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>446</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>447</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>449</v>
       </c>
       <c r="G18" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="37" t="s">
-        <v>130</v>
+      <c r="H18" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="48" t="s">
-        <v>445</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>446</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>447</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>448</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>449</v>
-      </c>
-      <c r="G19" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H19" s="33" t="s">
-        <v>68</v>
+      <c r="B19" s="49" t="s">
+        <v>450</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>451</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>452</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="G19" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H19" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="49" t="s">
-        <v>450</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>451</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>452</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>453</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>454</v>
-      </c>
-      <c r="G20" s="36" t="s">
-        <v>119</v>
+      <c r="B20" s="48" t="s">
+        <v>455</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>456</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>457</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>458</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>459</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H20" s="37" t="s">
         <v>130</v>
@@ -14636,51 +14546,25 @@
       <c r="A21" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="48" t="s">
-        <v>455</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>456</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>457</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>458</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>459</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>67</v>
+      <c r="B21" s="49" t="s">
+        <v>460</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>461</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>462</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>463</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>464</v>
+      </c>
+      <c r="G21" s="36" t="s">
+        <v>119</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="49" t="s">
-        <v>460</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>461</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>462</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>463</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>464</v>
-      </c>
-      <c r="G22" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -14689,6 +14573,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: resolve hackathon deadline visibility and add prize pool display
</commit_message>
<xml_diff>
--- a/Skillit_QA_Test_Report.xlsx
+++ b/Skillit_QA_Test_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/868af55b16e02466/Desktop/codes/extras/skillit-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_3F4C96BE085EF1FA77C6B918C4011D2484EEB7CA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA618568-A82F-4348-8418-A8C97102E25C}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="11_3F4C96BE085EF1FA77C6B918C4011D2484EEB7CA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E7D8E72-683E-4B0D-8716-79C3EB8628F5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3271" uniqueCount="1060">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="1060">
   <si>
     <t>SKILLIT</t>
   </si>
@@ -4730,7 +4730,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5253,102 +5253,24 @@
         <v>46</v>
       </c>
       <c r="B21" s="57" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>756</v>
+        <v>766</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>757</v>
+        <v>767</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>758</v>
+        <v>768</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>759</v>
-      </c>
-      <c r="G21" s="36" t="s">
-        <v>119</v>
+        <v>769</v>
+      </c>
+      <c r="G21" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="58" t="s">
-        <v>760</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>761</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>762</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>763</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>764</v>
-      </c>
-      <c r="G22" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H22" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="57" t="s">
-        <v>765</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>766</v>
-      </c>
-      <c r="D23" s="31" t="s">
-        <v>767</v>
-      </c>
-      <c r="E23" s="31" t="s">
-        <v>768</v>
-      </c>
-      <c r="F23" s="31" t="s">
-        <v>769</v>
-      </c>
-      <c r="G23" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H23" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="58" t="s">
-        <v>770</v>
-      </c>
-      <c r="C24" s="34" t="s">
-        <v>771</v>
-      </c>
-      <c r="D24" s="35" t="s">
-        <v>772</v>
-      </c>
-      <c r="E24" s="35" t="s">
-        <v>773</v>
-      </c>
-      <c r="F24" s="35" t="s">
-        <v>774</v>
-      </c>
-      <c r="G24" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H24" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -5362,7 +5284,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5572,23 +5494,23 @@
       <c r="A9" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="60" t="s">
-        <v>805</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>806</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>807</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>808</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>809</v>
-      </c>
-      <c r="G9" s="36" t="s">
-        <v>119</v>
+      <c r="B9" s="61" t="s">
+        <v>810</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>811</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>812</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>813</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>814</v>
+      </c>
+      <c r="G9" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H9" s="37" t="s">
         <v>130</v>
@@ -5599,19 +5521,19 @@
         <v>48</v>
       </c>
       <c r="B10" s="61" t="s">
-        <v>810</v>
+        <v>820</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>811</v>
+        <v>821</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>812</v>
+        <v>822</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>814</v>
+        <v>824</v>
       </c>
       <c r="G10" s="32" t="s">
         <v>67</v>
@@ -5625,22 +5547,22 @@
         <v>48</v>
       </c>
       <c r="B11" s="60" t="s">
-        <v>815</v>
+        <v>825</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>817</v>
+        <v>827</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>818</v>
+        <v>828</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>819</v>
-      </c>
-      <c r="G11" s="36" t="s">
-        <v>119</v>
+        <v>829</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H11" s="37" t="s">
         <v>130</v>
@@ -5651,19 +5573,19 @@
         <v>48</v>
       </c>
       <c r="B12" s="61" t="s">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>823</v>
+        <v>833</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>824</v>
+        <v>834</v>
       </c>
       <c r="G12" s="32" t="s">
         <v>67</v>
@@ -5677,19 +5599,19 @@
         <v>48</v>
       </c>
       <c r="B13" s="60" t="s">
-        <v>825</v>
+        <v>835</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>826</v>
+        <v>836</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>827</v>
+        <v>837</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>828</v>
+        <v>838</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>829</v>
+        <v>839</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>67</v>
@@ -5702,20 +5624,20 @@
       <c r="A14" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="61" t="s">
-        <v>830</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>831</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>832</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>833</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>834</v>
+      <c r="B14" s="60" t="s">
+        <v>845</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>846</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>847</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>848</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>849</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>67</v>
@@ -5729,19 +5651,19 @@
         <v>48</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>835</v>
+        <v>855</v>
       </c>
       <c r="C15" s="30" t="s">
-        <v>836</v>
+        <v>856</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>837</v>
+        <v>857</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>838</v>
+        <v>858</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>839</v>
+        <v>859</v>
       </c>
       <c r="G15" s="32" t="s">
         <v>67</v>
@@ -5755,22 +5677,22 @@
         <v>48</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>840</v>
+        <v>860</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>841</v>
+        <v>861</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>842</v>
+        <v>862</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>843</v>
+        <v>863</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>844</v>
-      </c>
-      <c r="G16" s="36" t="s">
-        <v>119</v>
+        <v>864</v>
+      </c>
+      <c r="G16" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H16" s="37" t="s">
         <v>130</v>
@@ -5780,155 +5702,25 @@
       <c r="A17" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="60" t="s">
-        <v>845</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>846</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>847</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>848</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>849</v>
+      <c r="B17" s="61" t="s">
+        <v>870</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>871</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>872</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>873</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>874</v>
       </c>
       <c r="G17" s="32" t="s">
         <v>67</v>
       </c>
       <c r="H17" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="61" t="s">
-        <v>850</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>851</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>852</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>853</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>854</v>
-      </c>
-      <c r="G18" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H18" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="60" t="s">
-        <v>855</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>856</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>857</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>858</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>859</v>
-      </c>
-      <c r="G19" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H19" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="61" t="s">
-        <v>860</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>861</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>862</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>863</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>864</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="60" t="s">
-        <v>865</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>866</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>867</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>868</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>869</v>
-      </c>
-      <c r="G21" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" s="61" t="s">
-        <v>870</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>871</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>872</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>873</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>874</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -14024,7 +13816,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14286,46 +14078,46 @@
       <c r="A11" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="49" t="s">
-        <v>410</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>411</v>
-      </c>
-      <c r="D11" s="35" t="s">
-        <v>412</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>413</v>
-      </c>
-      <c r="F11" s="35" t="s">
-        <v>414</v>
-      </c>
-      <c r="G11" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H11" s="33" t="s">
-        <v>68</v>
+      <c r="B11" s="48" t="s">
+        <v>415</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>416</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>417</v>
+      </c>
+      <c r="E11" s="31" t="s">
+        <v>418</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>419</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="48" t="s">
-        <v>415</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>416</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>417</v>
-      </c>
-      <c r="E12" s="31" t="s">
-        <v>418</v>
-      </c>
-      <c r="F12" s="31" t="s">
-        <v>419</v>
+      <c r="B12" s="49" t="s">
+        <v>420</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>421</v>
+      </c>
+      <c r="D12" s="35" t="s">
+        <v>422</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>423</v>
+      </c>
+      <c r="F12" s="35" t="s">
+        <v>424</v>
       </c>
       <c r="G12" s="32" t="s">
         <v>67</v>
@@ -14338,20 +14130,20 @@
       <c r="A13" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="49" t="s">
-        <v>420</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>421</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>422</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>423</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>424</v>
+      <c r="B13" s="48" t="s">
+        <v>425</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>426</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>427</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>428</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>429</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>67</v>
@@ -14364,72 +14156,72 @@
       <c r="A14" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="48" t="s">
-        <v>425</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>426</v>
-      </c>
-      <c r="D14" s="31" t="s">
-        <v>427</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>428</v>
-      </c>
-      <c r="F14" s="31" t="s">
-        <v>429</v>
+      <c r="B14" s="49" t="s">
+        <v>430</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>431</v>
+      </c>
+      <c r="D14" s="35" t="s">
+        <v>432</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="F14" s="35" t="s">
+        <v>434</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H14" s="37" t="s">
-        <v>130</v>
+      <c r="H14" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="49" t="s">
-        <v>430</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>431</v>
-      </c>
-      <c r="D15" s="35" t="s">
-        <v>432</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>433</v>
-      </c>
-      <c r="F15" s="35" t="s">
-        <v>434</v>
+      <c r="B15" s="48" t="s">
+        <v>435</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>436</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>437</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>438</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>439</v>
       </c>
       <c r="G15" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="33" t="s">
-        <v>68</v>
+      <c r="H15" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="48" t="s">
-        <v>435</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>436</v>
-      </c>
-      <c r="D16" s="31" t="s">
-        <v>437</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>438</v>
-      </c>
-      <c r="F16" s="31" t="s">
-        <v>439</v>
+      <c r="B16" s="49" t="s">
+        <v>440</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>441</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>442</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>443</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>444</v>
       </c>
       <c r="G16" s="32" t="s">
         <v>67</v>
@@ -14442,26 +14234,26 @@
       <c r="A17" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="49" t="s">
-        <v>440</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>441</v>
-      </c>
-      <c r="D17" s="35" t="s">
-        <v>442</v>
-      </c>
-      <c r="E17" s="35" t="s">
-        <v>443</v>
-      </c>
-      <c r="F17" s="35" t="s">
-        <v>444</v>
+      <c r="B17" s="48" t="s">
+        <v>445</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>446</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>447</v>
+      </c>
+      <c r="E17" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>449</v>
       </c>
       <c r="G17" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="37" t="s">
-        <v>130</v>
+      <c r="H17" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14469,102 +14261,24 @@
         <v>40</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="G18" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="49" t="s">
-        <v>450</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>451</v>
-      </c>
-      <c r="D19" s="35" t="s">
-        <v>452</v>
-      </c>
-      <c r="E19" s="35" t="s">
-        <v>453</v>
-      </c>
-      <c r="F19" s="35" t="s">
-        <v>454</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H19" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="48" t="s">
-        <v>455</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>456</v>
-      </c>
-      <c r="D20" s="31" t="s">
-        <v>457</v>
-      </c>
-      <c r="E20" s="31" t="s">
-        <v>458</v>
-      </c>
-      <c r="F20" s="31" t="s">
-        <v>459</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="49" t="s">
-        <v>460</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>461</v>
-      </c>
-      <c r="D21" s="35" t="s">
-        <v>462</v>
-      </c>
-      <c r="E21" s="35" t="s">
-        <v>463</v>
-      </c>
-      <c r="F21" s="35" t="s">
-        <v>464</v>
-      </c>
-      <c r="G21" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="37" t="s">
+      <c r="H18" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -14579,7 +14293,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14711,23 +14425,23 @@
       <c r="A6" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="52" t="s">
-        <v>480</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>481</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>482</v>
-      </c>
-      <c r="E6" s="35" t="s">
-        <v>483</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>484</v>
-      </c>
-      <c r="G6" s="36" t="s">
-        <v>119</v>
+      <c r="B6" s="51" t="s">
+        <v>485</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>486</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>487</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>488</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>489</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H6" s="37" t="s">
         <v>130</v>
@@ -14737,52 +14451,52 @@
       <c r="A7" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="51" t="s">
-        <v>485</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>486</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>487</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>488</v>
-      </c>
-      <c r="F7" s="31" t="s">
-        <v>489</v>
+      <c r="B7" s="52" t="s">
+        <v>490</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>491</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>492</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>493</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>494</v>
       </c>
       <c r="G7" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="37" t="s">
-        <v>130</v>
+      <c r="H7" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="52" t="s">
-        <v>490</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>491</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>492</v>
-      </c>
-      <c r="E8" s="35" t="s">
-        <v>493</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>494</v>
+      <c r="B8" s="51" t="s">
+        <v>495</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>497</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>498</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>499</v>
       </c>
       <c r="G8" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="33" t="s">
-        <v>68</v>
+      <c r="H8" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14790,25 +14504,25 @@
         <v>42</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="G9" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H9" s="37" t="s">
-        <v>130</v>
+      <c r="H9" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14816,22 +14530,22 @@
         <v>42</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>502</v>
+        <v>522</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>503</v>
+        <v>523</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>504</v>
-      </c>
-      <c r="G10" s="36" t="s">
-        <v>119</v>
+        <v>524</v>
+      </c>
+      <c r="G10" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H10" s="37" t="s">
         <v>130</v>
@@ -14842,25 +14556,25 @@
         <v>42</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>505</v>
+        <v>525</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>506</v>
+        <v>526</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>507</v>
+        <v>527</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>508</v>
+        <v>528</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>509</v>
+        <v>529</v>
       </c>
       <c r="G11" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H11" s="33" t="s">
-        <v>68</v>
+      <c r="H11" s="37" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14868,22 +14582,22 @@
         <v>42</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>510</v>
+        <v>530</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>511</v>
+        <v>531</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>512</v>
+        <v>532</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>513</v>
+        <v>533</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>514</v>
-      </c>
-      <c r="G12" s="36" t="s">
-        <v>119</v>
+        <v>534</v>
+      </c>
+      <c r="G12" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H12" s="37" t="s">
         <v>130</v>
@@ -14894,258 +14608,50 @@
         <v>42</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>515</v>
+        <v>535</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>516</v>
+        <v>536</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>517</v>
+        <v>537</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>518</v>
+        <v>538</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>519</v>
-      </c>
-      <c r="G13" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H13" s="37" t="s">
-        <v>130</v>
+        <v>539</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="33" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="52" t="s">
-        <v>520</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>521</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>522</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>523</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>524</v>
+      <c r="B14" s="51" t="s">
+        <v>555</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>556</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>557</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>559</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>67</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="51" t="s">
-        <v>525</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>526</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>527</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>528</v>
-      </c>
-      <c r="F15" s="31" t="s">
-        <v>529</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H15" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="52" t="s">
-        <v>530</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>531</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>532</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>533</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>534</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H16" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>535</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>536</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>537</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>538</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>539</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H17" s="33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="52" t="s">
-        <v>540</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>541</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>542</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>543</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>544</v>
-      </c>
-      <c r="G18" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H18" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>545</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>546</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>547</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>548</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>549</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H19" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="52" t="s">
-        <v>550</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>551</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>552</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>553</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>554</v>
-      </c>
-      <c r="G20" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>555</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>556</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>557</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>558</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>559</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="52" t="s">
-        <v>560</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>561</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>562</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>563</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>564</v>
-      </c>
-      <c r="G22" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>
@@ -15159,7 +14665,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -15655,23 +15161,23 @@
       <c r="A20" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="55" t="s">
-        <v>650</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>651</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>652</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>653</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>654</v>
-      </c>
-      <c r="G20" s="36" t="s">
-        <v>119</v>
+      <c r="B20" s="54" t="s">
+        <v>655</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>656</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>657</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>658</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>659</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="H20" s="37" t="s">
         <v>130</v>
@@ -15681,51 +15187,25 @@
       <c r="A21" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="54" t="s">
-        <v>655</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>656</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>657</v>
-      </c>
-      <c r="E21" s="31" t="s">
-        <v>658</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>659</v>
+      <c r="B21" s="55" t="s">
+        <v>660</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>661</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>662</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>663</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>664</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>67</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="55" t="s">
-        <v>660</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>661</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>662</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>663</v>
-      </c>
-      <c r="F22" s="35" t="s">
-        <v>664</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" s="37" t="s">
         <v>130</v>
       </c>
     </row>

</xml_diff>